<commit_message>
Done Chapter 4 and 5
</commit_message>
<xml_diff>
--- a/Test Cases And Rules.xlsx
+++ b/Test Cases And Rules.xlsx
@@ -14,10 +14,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={c84cfd45-575a-4408-aecb-7b2c75914c1f}</author>
+    <author>tc={ff5f7d82-cd3f-4572-94ba-4d35e34317a9}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{c84cfd45-575a-4408-aecb-7b2c75914c1f}" ref="A1">
+    <comment authorId="0" xr:uid="{ff5f7d82-cd3f-4572-94ba-4d35e34317a9}" ref="A1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="85">
   <si>
     <t>STT</t>
   </si>
@@ -75,70 +75,76 @@
     <t>Heavy Duty (Bảo hộ lao động)</t>
   </si>
   <si>
-    <t>1056.0</t>
-  </si>
-  <si>
-    <t>72.3</t>
-  </si>
-  <si>
-    <t>73.2</t>
-  </si>
-  <si>
-    <t>58.6</t>
+    <t>130.6</t>
+  </si>
+  <si>
+    <t>1165.0</t>
+  </si>
+  <si>
+    <t>85.3</t>
+  </si>
+  <si>
+    <t>86.1</t>
+  </si>
+  <si>
+    <t>82.9</t>
   </si>
   <si>
     <t>Delicates (Áo sơ mi lụa)</t>
   </si>
   <si>
-    <t>387.0</t>
-  </si>
-  <si>
-    <t>33.8</t>
+    <t>38.1</t>
+  </si>
+  <si>
+    <t>452.0</t>
   </si>
   <si>
     <t>Mixed Fabric (Đồ mặc nhà)</t>
   </si>
   <si>
-    <t>700.0</t>
+    <t>80.0</t>
+  </si>
+  <si>
+    <t>883.0</t>
   </si>
   <si>
     <t>50.0</t>
   </si>
   <si>
-    <t>40.0</t>
+    <t>46.7</t>
   </si>
   <si>
     <t>Baby Care (Đồ trẻ em)</t>
   </si>
   <si>
+    <t>82.5</t>
+  </si>
+  <si>
+    <t>631.0</t>
+  </si>
+  <si>
+    <t>45.8</t>
+  </si>
+  <si>
+    <t>45.4</t>
+  </si>
+  <si>
+    <t>Duvet (Chăn mền)</t>
+  </si>
+  <si>
     <t>91.7</t>
   </si>
   <si>
-    <t>474.0</t>
-  </si>
-  <si>
-    <t>46.4</t>
-  </si>
-  <si>
-    <t>47.7</t>
-  </si>
-  <si>
-    <t>48.8</t>
-  </si>
-  <si>
-    <t>Duvet (Chăn mền)</t>
-  </si>
-  <si>
-    <t>102.5</t>
-  </si>
-  <si>
-    <t>962.0</t>
-  </si>
-  <si>
-    <t>67.3</t>
-  </si>
-  <si>
-    <t>58.3</t>
+    <t>986.0</t>
+  </si>
+  <si>
+    <t>86.0</t>
+  </si>
+  <si>
+    <t>65.0</t>
+  </si>
+  <si>
+    <t>32.0</t>
   </si>
   <si>
     <t>NHÓM LUẬT</t>
@@ -287,7 +293,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+    <numFmt numFmtId="164" formatCode="d.m"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -478,7 +484,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="SGHPK 0905" id="{fab14d79-d227-45e2-a585-d944fab585cc}" providerId="google-sheets"/>
+  <x18tc:person displayName="SGHPK 0905" id="{e94c9f7b-3c1d-4970-93fb-057c73eafee8}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -678,7 +684,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A1" dT="2026-03-20T11:18:11.00" personId="{fab14d79-d227-45e2-a585-d944fab585cc}" id="{c84cfd45-575a-4408-aecb-7b2c75914c1f}" done="0">
+  <x18tc:threadedComment ref="A1" dT="2026-03-20T11:18:11.00" personId="{e94c9f7b-3c1d-4970-93fb-057c73eafee8}" id="{ff5f7d82-cd3f-4572-94ba-4d35e34317a9}" done="0">
     <x18tc:text xml:space="preserve">ví dụ nè</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -795,20 +801,20 @@
       <c r="F3" s="12">
         <v>1.0</v>
       </c>
-      <c r="G3" s="13">
-        <v>135.8</v>
-      </c>
-      <c r="H3" s="13" t="s">
+      <c r="G3" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="H3" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="I3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="K3" s="13" t="s">
+      <c r="J3" s="12" t="s">
         <v>17</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -816,7 +822,7 @@
         <v>2.0</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C4" s="12">
         <v>1.5</v>
@@ -830,20 +836,20 @@
       <c r="F4" s="12">
         <v>9.0</v>
       </c>
-      <c r="G4" s="13">
-        <v>56.2</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" s="13" t="s">
+      <c r="G4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="J4" s="13" t="s">
-        <v>20</v>
+      <c r="H4" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" s="13">
+        <v>46217.0</v>
+      </c>
+      <c r="J4" s="13">
+        <v>46217.0</v>
       </c>
       <c r="K4" s="13">
-        <v>28.1</v>
+        <v>46224.0</v>
       </c>
     </row>
     <row r="5">
@@ -851,7 +857,7 @@
         <v>3.0</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" s="12">
         <v>5.0</v>
@@ -865,20 +871,20 @@
       <c r="F5" s="12">
         <v>5.0</v>
       </c>
-      <c r="G5" s="13">
-        <v>90.0</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" s="13" t="s">
+      <c r="G5" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" s="13" t="s">
+      <c r="H5" s="12" t="s">
         <v>24</v>
+      </c>
+      <c r="I5" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="J5" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="6">
@@ -886,7 +892,7 @@
         <v>4.0</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C6" s="12">
         <v>3.5</v>
@@ -900,20 +906,20 @@
       <c r="F6" s="12">
         <v>8.0</v>
       </c>
-      <c r="G6" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="13" t="s">
+      <c r="G6" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="J6" s="13" t="s">
+      <c r="H6" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="K6" s="13" t="s">
+      <c r="I6" s="12" t="s">
         <v>30</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="7">
@@ -921,7 +927,7 @@
         <v>5.0</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C7" s="12">
         <v>9.0</v>
@@ -935,20 +941,20 @@
       <c r="F7" s="12">
         <v>4.0</v>
       </c>
-      <c r="G7" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="H7" s="13" t="s">
+      <c r="G7" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="H7" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="J7" s="13" t="s">
+      <c r="I7" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="K7" s="13" t="s">
-        <v>24</v>
+      <c r="J7" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -982,54 +988,54 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
       <c r="K1" s="4"/>
       <c r="L1" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
       <c r="C2" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L2" s="7"/>
     </row>
@@ -1038,37 +1044,37 @@
         <v>1.0</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G3" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="I3" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="H3" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>50</v>
-      </c>
       <c r="J3" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K3" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L3" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
@@ -1076,37 +1082,37 @@
         <v>2.0</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G4" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="H4" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="I4" s="12" t="s">
-        <v>56</v>
-      </c>
       <c r="J4" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5">
@@ -1114,37 +1120,37 @@
         <v>3.0</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6">
@@ -1152,37 +1158,37 @@
         <v>4.0</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C6" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="J6" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="H6" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="12" t="s">
-        <v>63</v>
-      </c>
       <c r="K6" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7">
@@ -1190,37 +1196,37 @@
         <v>5.0</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E7" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="H7" s="12" t="s">
-        <v>54</v>
-      </c>
       <c r="I7" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J7" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K7" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="L7" s="10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8">
@@ -1228,37 +1234,37 @@
         <v>6.0</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C8" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="I8" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="K8" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="E8" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="H8" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="I8" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="J8" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="K8" s="12" t="s">
-        <v>60</v>
-      </c>
       <c r="L8" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9">
@@ -1266,37 +1272,37 @@
         <v>7.0</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J9" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10">
@@ -1304,37 +1310,37 @@
         <v>8.0</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11">
@@ -1342,37 +1348,37 @@
         <v>9.0</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I11" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J11" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K11" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12">
@@ -1380,37 +1386,37 @@
         <v>10.0</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J12" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K12" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13">
@@ -1418,37 +1424,37 @@
         <v>11.0</v>
       </c>
       <c r="B13" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="G13" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C13" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>69</v>
-      </c>
       <c r="H13" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J13" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K13" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14">
@@ -1456,37 +1462,37 @@
         <v>12.0</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I14" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K14" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15">
@@ -1494,37 +1500,37 @@
         <v>13.0</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16">
@@ -1532,37 +1538,37 @@
         <v>14.0</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I16" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J16" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K16" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17">
@@ -1570,46 +1576,46 @@
         <v>15.0</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H17" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I17" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J17" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:F1"/>
     <mergeCell ref="G1:K1"/>
     <mergeCell ref="L1:L2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:F1"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>